<commit_message>
Complemented descriptive statistics with frequency analysis
</commit_message>
<xml_diff>
--- a/src/variance/napire24-variance-overview.xlsx
+++ b/src/variance/napire24-variance-overview.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julfrat\Workspace\napire2024\src\variance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12A93FD6-77BA-4F4D-898D-66FF190D009E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD15F7A0-A561-4BAF-A87F-A2383574DB58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="42330" yWindow="-14160" windowWidth="24975" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Common Responses and Effects" sheetId="1" r:id="rId1"/>
@@ -625,18 +625,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Lead decided enough thime spent: Disagree, Lead decided enough time wasted: Disagree, Team agreed enough time wasted: Disagree, Itching to start implementation: no opinion (95% CI)	</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">
 </t>
     </r>
@@ -933,6 +921,9 @@
   </si>
   <si>
     <t>scheduled end: agree / lead decided enough time spent: disagree / Lead decided enough time wasted: disagree / Team agreed enough time wasted: disagree / Team agreed time pressure: agree / starting real work: no opinion / itching to start implementation: no opinion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lead decided enough time spent: Disagree, Lead decided enough time wasted: Disagree, Team agreed enough time wasted: Disagree, Itching to start implementation: no opinion (95% CI)	</t>
   </si>
 </sst>
 </file>
@@ -1461,7 +1452,7 @@
         <v>105</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>28</v>
@@ -1514,7 +1505,7 @@
         <v>106</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>29</v>
@@ -1561,7 +1552,7 @@
         <v>105</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>27</v>
@@ -1608,7 +1599,7 @@
         <v>107</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>60</v>
@@ -1652,7 +1643,7 @@
         <v>35</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>61</v>
@@ -1678,7 +1669,7 @@
         <v>108</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>86</v>
@@ -1725,7 +1716,7 @@
         <v>109</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>64</v>
@@ -1825,7 +1816,7 @@
         <v>99</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I10" s="1" t="s">
         <v>100</v>
@@ -1869,7 +1860,7 @@
         <v>129</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>104</v>
@@ -1916,7 +1907,7 @@
         <v>112</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I12" s="1" t="s">
         <v>72</v>
@@ -1969,7 +1960,7 @@
         <v>113</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>91</v>
@@ -2042,7 +2033,7 @@
         <v>135</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>80</v>
@@ -2086,10 +2077,10 @@
         <v>90</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="H16" s="10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="I16" s="1" t="s">
         <v>102</v>
@@ -2098,19 +2089,19 @@
         <v>119</v>
       </c>
       <c r="L16" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="N16" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="N16" s="9" t="s">
+      <c r="P16" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="P16" s="9" t="s">
+      <c r="R16" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="R16" s="9" t="s">
+      <c r="T16" s="9" t="s">
         <v>141</v>
-      </c>
-      <c r="T16" s="9" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="17" spans="1:20" ht="144" x14ac:dyDescent="0.3">
@@ -2133,7 +2124,7 @@
         <v>114</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I17" s="1" t="s">
         <v>83</v>

</xml_diff>